<commit_message>
delete code and update feature list
</commit_message>
<xml_diff>
--- a/url_features_table.xlsx
+++ b/url_features_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\URL-Phishing-Detection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE4641D-9AE8-415C-A0C4-8584948D911E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86226964-3A49-4A42-A53B-EC61343C3986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="400">
   <si>
     <t>No</t>
   </si>
@@ -1040,13 +1040,205 @@
   </si>
   <si>
     <t>Malicious_URL_Detection_and_Categorization_Using_Machine_Learning_Techniques</t>
+  </si>
+  <si>
+    <t>LengthOfURL</t>
+  </si>
+  <si>
+    <t>DomainLengthOfURL</t>
+  </si>
+  <si>
+    <t>Having_Path</t>
+  </si>
+  <si>
+    <t>ShannonEntropy</t>
+  </si>
+  <si>
+    <t>KolmogorovComplexity</t>
+  </si>
+  <si>
+    <t>HexPatternCnt</t>
+  </si>
+  <si>
+    <t>Base64PatternCnt</t>
+  </si>
+  <si>
+    <t>Average_Word</t>
+  </si>
+  <si>
+    <t>Base64_Pattern_Cnt</t>
+  </si>
+  <si>
+    <t>Check_EXE</t>
+  </si>
+  <si>
+    <t>Check_IP_HostName</t>
+  </si>
+  <si>
+    <t>Count_%</t>
+  </si>
+  <si>
+    <t>Count_/</t>
+  </si>
+  <si>
+    <t>Count_All_Functions</t>
+  </si>
+  <si>
+    <t>Count_Digit</t>
+  </si>
+  <si>
+    <t>Count_Dir</t>
+  </si>
+  <si>
+    <t>Count_Dot</t>
+  </si>
+  <si>
+    <t>Count_Embed_Domain</t>
+  </si>
+  <si>
+    <t>Orijinal</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>Character _Repetition</t>
+  </si>
+  <si>
+    <t>Count_Letter</t>
+  </si>
+  <si>
+    <t>Count_Path_Slash</t>
+  </si>
+  <si>
+    <t>Count_Search</t>
+  </si>
+  <si>
+    <t>Count_Symbols</t>
+  </si>
+  <si>
+    <t>Count-Http</t>
+  </si>
+  <si>
+    <t>Count-Https</t>
+  </si>
+  <si>
+    <t>Count_www</t>
+  </si>
+  <si>
+    <t>Dash_Char_Count</t>
+  </si>
+  <si>
+    <t>Delimiter_Count</t>
+  </si>
+  <si>
+    <t>Digit_Alphabet_Ratio</t>
+  </si>
+  <si>
+    <t>Digits_in_Domain_Name</t>
+  </si>
+  <si>
+    <t>Digits_in_Host</t>
+  </si>
+  <si>
+    <t>Dist_Digit_Alphabet</t>
+  </si>
+  <si>
+    <t>Dist_Word_Based</t>
+  </si>
+  <si>
+    <t>Domain_Name</t>
+  </si>
+  <si>
+    <t>Domain_Length_Of_URL</t>
+  </si>
+  <si>
+    <t>Domain_URL_Ratio</t>
+  </si>
+  <si>
+    <t>Double_Slash_Count</t>
+  </si>
+  <si>
+    <t>File_Extension</t>
+  </si>
+  <si>
+    <t>FTP_Used</t>
+  </si>
+  <si>
+    <t>Hash_Char_Count</t>
+  </si>
+  <si>
+    <t>Hex_Pattern_Cnt</t>
+  </si>
+  <si>
+    <t>Host_Length</t>
+  </si>
+  <si>
+    <t>Host_Precense_Of_Digit</t>
+  </si>
+  <si>
+    <t>IP_Address</t>
+  </si>
+  <si>
+    <t>Kolmogorov_Complexity</t>
+  </si>
+  <si>
+    <t>Length_OfURL</t>
+  </si>
+  <si>
+    <t>Longest_Word</t>
+  </si>
+  <si>
+    <t>Longest_Word_in_Hostname</t>
+  </si>
+  <si>
+    <t>Longest/Shortest _Word_Length</t>
+  </si>
+  <si>
+    <t>Numeric_Char_Count</t>
+  </si>
+  <si>
+    <t>Path_Length</t>
+  </si>
+  <si>
+    <t>Percent_Char_Count</t>
+  </si>
+  <si>
+    <t>Port_Number</t>
+  </si>
+  <si>
+    <t>Query_Length</t>
+  </si>
+  <si>
+    <t>Semi_Col_Count</t>
+  </si>
+  <si>
+    <t>Shortest_Word</t>
+  </si>
+  <si>
+    <t>Special_Char_Alphabet_Ratio</t>
+  </si>
+  <si>
+    <t>STD_of_Words_Length</t>
+  </si>
+  <si>
+    <t>Tld_Length</t>
+  </si>
+  <si>
+    <t>Uppercase_Lowercase_Ratio</t>
+  </si>
+  <si>
+    <t>URL_Without_www</t>
+  </si>
+  <si>
+    <t>Short_Url</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1078,8 +1270,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+      <charset val="162"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF6A9955"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+      <charset val="162"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1089,6 +1295,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1129,7 +1341,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1162,6 +1374,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4481,393 +4704,658 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B66078BF-7097-A04E-85DC-24CEE7935F32}">
-  <dimension ref="A1:A76"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" customWidth="1"/>
+    <col min="7" max="7" width="39" style="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
+        <v>354</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="E2" s="4" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>342</v>
+      </c>
+      <c r="E3" t="s">
+        <v>344</v>
+      </c>
+      <c r="G3" s="15"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="E4" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="G4" s="13"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="E5" t="s">
+        <v>345</v>
+      </c>
+      <c r="G5" s="13"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="E6" t="s">
+        <v>346</v>
+      </c>
+      <c r="G6" s="13"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="G7" s="13"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>156</v>
+      </c>
+      <c r="G8" s="12"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+      <c r="E9" t="s">
+        <v>160</v>
+      </c>
+      <c r="G9" s="13"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>348</v>
+      </c>
+      <c r="G10" s="13"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+      <c r="E11" t="s">
+        <v>150</v>
+      </c>
+      <c r="G11" s="13"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>152</v>
+      </c>
+      <c r="E12" t="s">
+        <v>152</v>
+      </c>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>158</v>
+      </c>
+      <c r="E13" t="s">
+        <v>158</v>
+      </c>
+      <c r="G13" s="13"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="E14" t="s">
+        <v>154</v>
+      </c>
+      <c r="G14" s="13"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="E15" t="s">
+        <v>349</v>
+      </c>
+      <c r="G15" s="13"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="E16" t="s">
+        <v>350</v>
+      </c>
+      <c r="G16" s="13"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="E17" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="G17" s="13"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="E18" t="s">
+        <v>352</v>
+      </c>
+      <c r="G18" s="12"/>
+    </row>
+    <row r="19" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="E19" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="G19" s="13"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="E20" t="s">
+        <v>357</v>
+      </c>
+      <c r="G20" s="13"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="E21" t="s">
+        <v>358</v>
+      </c>
+      <c r="G21" s="13"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="E22" t="s">
+        <v>359</v>
+      </c>
+      <c r="G22" s="13"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="E23" t="s">
+        <v>360</v>
+      </c>
+      <c r="G23" s="13"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="E24" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="G24" s="13"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="E25" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="G25" s="12"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E26" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="G26" s="13"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E27" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E28" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E29" s="4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E30" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="E31" s="4" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E32" s="4" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E33" s="4" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E34" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="E35" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="E36" s="4" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="E38" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
+      <c r="E39" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="E40" s="4" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="E41" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="E42" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" s="4" t="s">
+      <c r="E43" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>341</v>
+      </c>
+      <c r="E45" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="4" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="E46" s="4" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+      <c r="E47" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" s="4" t="s">
+      <c r="E48" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+      <c r="E49" s="4" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>340</v>
+      </c>
+      <c r="E50" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" s="4" t="s">
+      <c r="E51" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="4" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
+      <c r="E53" s="4" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A54" s="4" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
+      <c r="E54" s="4" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+      <c r="E55" s="4" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" s="4" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" s="4" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="E56" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+      <c r="E57" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
+      <c r="E58" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="4" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" s="4" t="s">
+      <c r="E59" s="4" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="4" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+      <c r="E60" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+      <c r="E61" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" s="4" t="s">
+      <c r="E62" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>339</v>
+      </c>
+      <c r="E63" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="4" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" s="4" t="s">
+      <c r="E64" s="4" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="4" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+      <c r="E65" s="4" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" s="4" t="s">
+      <c r="E66" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="4" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" s="4" t="s">
+      <c r="E67" s="4" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="4" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" s="4" t="s">
+      <c r="E68" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="4" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" s="4" t="s">
+      <c r="E69" s="4" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="4" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+      <c r="E70" s="4" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" s="4" t="s">
+      <c r="E71" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="4" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+      <c r="E72" s="4" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" s="4" t="s">
+      <c r="E73" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="4" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+      <c r="E74" s="4" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" s="4" t="s">
+      <c r="E75" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="4" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" s="4" t="s">
+      <c r="E76" s="4" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="4" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" s="4" t="s">
-        <v>196</v>
+      <c r="E77" s="4" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A77">
+    <sortCondition ref="A2:A77"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>